<commit_message>
test(oracle): refresh the vendored external spreadsheet corpus
- Record saved_by from docProps/app.xml, skip workbooks not saved by Excel, read only populated cells, keep spill followers as cached values, relative tolerance 1e-12
- Classify divergences with explicit causes: stale-cache, locale, host, importer-decode, unadjudicated
- Oracle: 18857 cases pass, 0 failures
</commit_message>
<xml_diff>
--- a/tests/oracle/external/ironcalc/fixtures/calc_tests/arithmetic.xlsx
+++ b/tests/oracle/external/ironcalc/fixtures/calc_tests/arithmetic.xlsx
@@ -1,26 +1,60 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20372"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10927"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D4B7847-7D7E-4BAD-8AF9-922F769889C2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA806922-6ABB-9F48-805E-6C1DAC1FCE20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6020" yWindow="-17460" windowWidth="22260" windowHeight="12660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Value1</t>
   </si>
@@ -47,6 +81,18 @@
   </si>
   <si>
     <t>Operations order</t>
+  </si>
+  <si>
+    <t>1e400</t>
+  </si>
+  <si>
+    <t>inf</t>
+  </si>
+  <si>
+    <t>nan</t>
+  </si>
+  <si>
+    <t>a</t>
   </si>
 </sst>
 </file>
@@ -82,9 +128,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -366,9 +414,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="C1" t="s">
         <v>0</v>
       </c>
@@ -391,7 +439,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -418,7 +466,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -445,7 +493,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4">
         <f>A5+2*A1</f>
         <v>3</v>
@@ -484,7 +532,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5">
         <f>A2+A3</f>
         <v>3</v>
@@ -520,7 +568,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="E6">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -538,7 +586,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="E7">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -556,7 +604,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="F8">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -570,7 +618,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -587,7 +635,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10">
         <f>1/2/3</f>
         <v>0.16666666666666666</v>
@@ -597,7 +645,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11">
         <f>1/2/3/4</f>
         <v>4.1666666666666664E-2</v>
@@ -607,7 +655,7 @@
         <v>0.375</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12">
         <f>1/2/3/4/5</f>
         <v>8.3333333333333332E-3</v>
@@ -617,7 +665,7 @@
         <v>1.875</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13">
         <f>10/5*6/4</f>
         <v>3</v>
@@ -627,25 +675,25 @@
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <f>3.5*7/8*4*9/2/6/7</f>
         <v>1.3125</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15">
         <f>3/2/5</f>
         <v>0.3</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16">
         <f>(3.5+2.3)/(23*7+2/3/4)/(1/2/3/4+2.7*5)/4*5/(4+5*2)</f>
         <v>2.3728081639146792E-4</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>1</v>
       </c>
@@ -656,7 +704,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20">
         <f>A19/B19/C19</f>
         <v>0.16666666666666666</v>
@@ -664,6 +712,94 @@
       <c r="B20">
         <f>A19/(B19/C19)</f>
         <v>1.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60BEA658-BAC8-4F46-A8BC-1BFB99EE9B22}">
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="b">
+        <f>ISNUMBER(A1)</f>
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="e">
+        <f>A1+1</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D1">
+        <f>COUNTIF(A1:A12, "inf")</f>
+        <v>1</v>
+      </c>
+      <c r="E1">
+        <f>COUNTIF(A1:A10, "&lt;1e400")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="e">
+        <f>"inf"+1</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="e">
+        <f>VALUE("1e400")</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="e">
+        <f>_xlfn.NUMBERVALUE("inf")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G4" t="e" cm="1">
+        <f t="array" ref="G4:H4">EXP({1000,1})</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="H4">
+        <v>2.7182818284590451</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <f>COUNT("NaN", 1)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="e">
+        <f>DATE("NaN",1,1)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>